<commit_message>
fix(pre-brd-unifier): apply the step 6 fix round
- decisions P2, P3, P6, P13 and N-2 (scoring and Excel export): one
  mapping for the Markdown chunks and the workbook; cell-map.json,
  export_xlsx.py, the reference workbook and the exporter tests
  updated
- triage, consistency and recheck fixes in SKILL.md, the README, the
  chunks and the framework notes; the inventory's source count is
  defined as distinct source links
- heading separators use colons; no em dashes
- exporter tests: 14 pass

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FSjNeYn9SPMZsYiE8dhLMu
</commit_message>
<xml_diff>
--- a/pre-brd-unifier/reference/PRE-BRD-v1.1.xlsx
+++ b/pre-brd-unifier/reference/PRE-BRD-v1.1.xlsx
@@ -54,210 +54,8 @@
 </workbook>
 </file>
 
-<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
-  <authors>
-    <author>M Shahin</author>
-  </authors>
-  <commentList>
-    <comment ref="B11" authorId="0" shapeId="0" xr:uid="{9E071E2A-CF96-4F40-B684-485E3D6F6C95}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <charset val="1"/>
-          </rPr>
-          <t>M Shahin:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <charset val="1"/>
-          </rPr>
-          <t xml:space="preserve">
-Source: Fortune Business Insights, Event Management Software Market (report 102611), 2025 — global EMS market USD 9.90B. https://www.fortunebusinessinsights.com/event-management-software-market-102611</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="B12" authorId="0" shapeId="0" xr:uid="{E7C5DE92-8516-4E5E-A3B8-C481AF894610}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <charset val="1"/>
-          </rPr>
-          <t>M Shahin:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <charset val="1"/>
-          </rPr>
-          <t xml:space="preserve">
-Source: Grand View Research (NA &gt;45% in 2024) and Fortune Business Insights (NA ~35% in 2025); 40% used as a midpoint. https://www.grandviewresearch.com/industry-analysis/event-management-software-market-report</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="B14" authorId="0" shapeId="0" xr:uid="{DF169AAA-9266-42BF-8F65-77F41F759CEB}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <charset val="1"/>
-          </rPr>
-          <t>M Shahin:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <charset val="1"/>
-          </rPr>
-          <t xml:space="preserve">
-EventHive assumption: share of the EMS market attributable to residential community / HOA / venue-amenity events (vs. corporate, conferences, concerts). Internal estimate — refine with primary research.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="B18" authorId="0" shapeId="0" xr:uid="{C9E22940-865C-4380-B170-366AED94B6BA}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <charset val="1"/>
-          </rPr>
-          <t>M Shahin:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <charset val="1"/>
-          </rPr>
-          <t xml:space="preserve">
-Source: Community Associations Institute (CAI) / iPropertyManagement, 2024 — ~370,000 community associations in the US. https://ipropertymanagement.com/research/hoa-statistics</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="B19" authorId="0" shapeId="0" xr:uid="{9907A8A3-1FE9-4AF8-9C10-D0B3EFAA2B39}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <charset val="1"/>
-          </rPr>
-          <t>M Shahin:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <charset val="1"/>
-          </rPr>
-          <t xml:space="preserve">
-EventHive assumption: ~8,000 are large-scale (&gt;1,000 homes) per CAI; 15% broadens to mid-size amenity-rich communities likely to buy event/venue software. Refine with segmentation research.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="B21" authorId="0" shapeId="0" xr:uid="{AD649284-6387-45E3-8FE1-3A176AAE3678}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <charset val="1"/>
-          </rPr>
-          <t>M Shahin:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <charset val="1"/>
-          </rPr>
-          <t xml:space="preserve">
-EventHive pricing assumption: ~$250/mo subscription = $3,000/yr per community for event/venue management software. Pricing input — NOT HOA resident dues. Validate against pilot pricing.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="B26" authorId="0" shapeId="0" xr:uid="{2785CD19-05B7-4420-93B7-556A348E80AF}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <charset val="1"/>
-          </rPr>
-          <t>M Shahin:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <charset val="1"/>
-          </rPr>
-          <t xml:space="preserve">
-EventHive assumption: share of US community-event TAM in EventHive's initial launch geography/segment (e.g. target states with high HOA density — FL, TX, CA, AZ). Refine to actual launch footprint.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="B28" authorId="0" shapeId="0" xr:uid="{433C9937-B9C1-4D57-A5C1-E62D204477E8}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <charset val="1"/>
-          </rPr>
-          <t>M Shahin:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <charset val="1"/>
-          </rPr>
-          <t xml:space="preserve">
-EventHive assumption: realistic share of SAM captured in first 1–3 years given sales capacity and competition. Refine with go-to-market plan.</t>
-        </r>
-      </text>
-    </comment>
-  </commentList>
-</comments>
-</file>
-
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3034" uniqueCount="756">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3034" uniqueCount="757">
   <si>
     <t>Page</t>
   </si>
@@ -1482,7 +1280,7 @@
     <t>TAM (Total Addressable Market)</t>
   </si>
   <si>
-    <t>The total demand for your product globally</t>
+    <t>The total demand for your product in the target segment and region, as sized in sections 1 to 3</t>
   </si>
   <si>
     <t>SAM (Serviceable Available Market)</t>
@@ -1497,7 +1295,7 @@
     <t>The realistic share of SAM you can capture initially</t>
   </si>
   <si>
-    <t>All event organizers worldwide</t>
+    <t>All event organizers in the target segment and region</t>
   </si>
   <si>
     <t>Event organizers in the MENA region</t>
@@ -1746,7 +1544,7 @@
     <t>brief</t>
   </si>
   <si>
-    <t>Identify all factors that might effect the product externally</t>
+    <t>Identify all factors that might affect the product externally</t>
   </si>
   <si>
     <t>Define whether the factor is Strength(S) or Weakness(W)</t>
@@ -1764,7 +1562,7 @@
     <t>Define whether the factor is Opportunity(O) or Threat(T)</t>
   </si>
   <si>
-    <t>Rate the factor effectivness or possibility to occur (week=0, Strong=5)</t>
+    <t>Rate how well the product's strategy responds to the factor, threats included (1=Poor, 5=Strong)</t>
   </si>
   <si>
     <t>IFAS</t>
@@ -2077,7 +1875,7 @@
     <t>Importance of the factor (from 0 to 1)</t>
   </si>
   <si>
-    <t>Rate internal performance on this factor (weak=0, Strong=5)</t>
+    <t>Rate internal performance on this factor (1=Poor, 5=Strong)</t>
   </si>
   <si>
     <t>All factor weights should = 1</t>
@@ -2338,7 +2136,7 @@
     <t>Objective Key Results (OKRs) Template with Sample</t>
   </si>
   <si>
-    <t>1. Top-Down (from US event-management-software market)</t>
+    <t>1. Top-down (from the relevant industry software market)</t>
   </si>
   <si>
     <t>Value</t>
@@ -2347,67 +2145,67 @@
     <t>Notes / source</t>
   </si>
   <si>
-    <t>Global EMS market (2025)</t>
+    <t>Global market (current year, in USD)</t>
   </si>
   <si>
     <t>Global event-management-software revenue, 2025</t>
   </si>
   <si>
-    <t>North America share of market</t>
+    <t>Region share of market</t>
   </si>
   <si>
     <t>NA share of global EMS (midpoint of cited 35–45%)</t>
   </si>
   <si>
-    <t>US EMS market (TAM, all segments)</t>
-  </si>
-  <si>
-    <t>= Global × NA share (US ≈ most of NA)</t>
-  </si>
-  <si>
-    <t>% relevant to community/residential events</t>
+    <t>Regional market (TAM, all segments)</t>
+  </si>
+  <si>
+    <t>= Global × region share</t>
+  </si>
+  <si>
+    <t>% relevant to the target segment</t>
   </si>
   <si>
     <t>EventHive assumption — community-event slice of total EMS</t>
   </si>
   <si>
-    <t>Serviceable TAM (community-event EMS, US)</t>
-  </si>
-  <si>
-    <t>Top-down TAM for EventHive's niche</t>
-  </si>
-  <si>
-    <t>2. Bottom-Up (from US HOA / community associations)</t>
-  </si>
-  <si>
-    <t>US community associations (HOAs)</t>
+    <t>Serviceable TAM (segment, region)</t>
+  </si>
+  <si>
+    <t>= Regional market × % relevant (top-down TAM for the niche)</t>
+  </si>
+  <si>
+    <t>2. Bottom-up (from addressable customer count)</t>
+  </si>
+  <si>
+    <t>Total addressable customers (universe)</t>
   </si>
   <si>
     <t>Total US HOAs/community associations (2024)</t>
   </si>
   <si>
-    <t>% addressable (mid/large, amenity-rich)</t>
+    <t>% addressable (right size / need)</t>
   </si>
   <si>
     <t>EventHive assumption — share with budget &amp; need</t>
   </si>
   <si>
-    <t>Addressable communities</t>
-  </si>
-  <si>
-    <t>= HOAs × addressable %</t>
-  </si>
-  <si>
-    <t>Annual software spend per community ($)</t>
+    <t>Addressable customers</t>
+  </si>
+  <si>
+    <t>= universe × addressable %</t>
+  </si>
+  <si>
+    <t>Annual software spend per customer (ARPU, in USD)</t>
   </si>
   <si>
     <t>EventHive ARPU assumption ($250/mo × 12)</t>
   </si>
   <si>
-    <t>Bottom-up TAM (addressable × ARPU)</t>
-  </si>
-  <si>
-    <t>Bottom-up serviceable market estimate</t>
+    <t>Bottom-up TAM</t>
+  </si>
+  <si>
+    <t>= addressable customers × ARPU</t>
   </si>
   <si>
     <t>3. TAM / SAM / SOM Summary</t>
@@ -2416,13 +2214,13 @@
     <t>Basis</t>
   </si>
   <si>
-    <t>TAM — US community-event software</t>
-  </si>
-  <si>
-    <t>Average of top-down ($198M) and bottom-up ($167M)</t>
-  </si>
-  <si>
-    <t>SAM — initial target geography/segment</t>
+    <t>TAM</t>
+  </si>
+  <si>
+    <t>= average of top-down and bottom-up TAM</t>
+  </si>
+  <si>
+    <t>SAM %</t>
   </si>
   <si>
     <t>% of TAM in launch footprint</t>
@@ -2434,7 +2232,7 @@
     <t>= TAM × SAM %</t>
   </si>
   <si>
-    <t>SOM — realistic capture (yr 1–3)</t>
+    <t>SOM %</t>
   </si>
   <si>
     <t>% of SAM captured early</t>
@@ -2752,10 +2550,10 @@
     <t>Sample (READ ONLY) — competitor landscape</t>
   </si>
   <si>
-    <t>TAM, SAM, SOM — sized two ways and cross-checked.
-Top-Down: start from the US event-management-software market (from industry reports), then narrow to the community/residential-events slice.
-Bottom-Up: addressable US HOAs/communities × annual software spend (ARPU).
-EventHive result (US): TAM ≈ $182M → SAM ≈ $46M → SOM ≈ $2.3M. See the Market Sizing tab for sourced inputs and formulas.</t>
+    <t>TAM, SAM, and SOM, sized two ways and cross-checked.
+Top-Down: start from the relevant industry software market (from industry reports), then narrow to the addressable slice.
+Bottom-Up: addressable customers × annual software spend (ARPU).
+See the Market Sizing tab for sourced inputs and formulas.</t>
   </si>
   <si>
     <t xml:space="preserve">Executive Comparison (With Top 5 products &amp; Empathy Map) - Sample READ ONLY </t>
@@ -2764,7 +2562,7 @@
     <t>Executive Comparison (With Top 5 products &amp; Empathy Map) - To be filled</t>
   </si>
   <si>
-    <t>EventHive — Market Sizing (US, gated/HOA communities) Sample - Read only</t>
+    <t>Market Sizing and Analysis</t>
   </si>
   <si>
     <t>Go / No-Go synthesis — aggregates the signals from all analysis tabs into a single recommendation.</t>
@@ -2900,6 +2698,9 @@
   </si>
   <si>
     <t>Go / No-Go synthesis. Aggregates the five signals (market attractiveness, problem/solution fit, feasibility, competitive risk, strategic fit) from the tabs above into a single weighted composite and recommendation. Generated on demand from the control panel; verifies all dependencies are filled before scoring.</t>
+  </si>
+  <si>
+    <t>Identify all factors that might affect the product internally</t>
   </si>
 </sst>
 </file>
@@ -7158,7 +6959,7 @@
     <row r="11" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A11" s="92"/>
       <c r="B11" s="61" t="s">
-        <v>400</v>
+        <v>756</v>
       </c>
       <c r="C11" s="61" t="s">
         <v>401</v>
@@ -9564,8 +9365,7 @@
         <v>741</v>
       </c>
       <c r="J6">
-        <f>IF(OR(COUNT(EFAS!E2:E6)&lt;5,COUNT(EFAS!D2:D6)&lt;5,SUM(EFAS!D2:D6)=0),0,1)</f>
-        <v>1</v>
+        <f>IF(OR(COUNT(EFAS!E2:E6)&lt;5,COUNT(EFAS!D2:D6)&lt;5,SUM(EFAS!D2:D6)=0,COUNTIF(EFAS!C2:C6,"O")=0,SUMIF(EFAS!C2:C6,"O",EFAS!D2:D6)=0),0,1)</f>
       </c>
     </row>
     <row r="7" spans="2:10" ht="20" customHeight="1" x14ac:dyDescent="0.35">
@@ -9581,8 +9381,7 @@
         <v>742</v>
       </c>
       <c r="J7">
-        <f>IF(OR(COUNT('IFAS '!E2:E5)&lt;4,COUNT('IFAS '!D2:D5)&lt;4,SUM('IFAS '!D2:D5)=0),0,1)</f>
-        <v>1</v>
+        <f>IF(OR(COUNT('IFAS '!E2:E5)&lt;4,COUNT('IFAS '!D2:D5)&lt;4,SUM('IFAS '!D2:D5)=0,COUNTIF('IFAS '!C2:C5,"S")=0,SUMIF('IFAS '!C2:C5,"S",'IFAS '!D2:D5)=0),0,1)</f>
       </c>
     </row>
     <row r="8" spans="2:10" ht="20" customHeight="1" x14ac:dyDescent="0.35">
@@ -9703,11 +9502,10 @@
         <v>722</v>
       </c>
       <c r="C18" s="266" t="str">
-        <f>"EFAS opportunity strength "&amp;TEXT(SUM(EFAS!F2:F4)/SUM(EFAS!D2:D4),"0.0")&amp;"/5"</f>
-        <v>EFAS opportunity strength 4.1/5</v>
+        <f>IF(SUMIF(EFAS!C2:C6,"O",EFAS!D2:D6)=0,"[NEEDS CLARIFICATION: EFAS opportunities have zero total weight]","EFAS opportunity rating "&amp;TEXT(SUMIF(EFAS!C2:C6,"O",EFAS!F2:F6)/SUMIF(EFAS!C2:C6,"O",EFAS!D2:D6),"0.0")&amp;"/5")</f>
       </c>
       <c r="D18" s="267" t="str">
-        <f>IF($C$8=0,"—",ROUND(SUM(EFAS!F2:F4)/SUM(EFAS!D2:D4),1))</f>
+        <f>IF($C$8=0,"—",ROUND(SUMIF(EFAS!C2:C6,"O",EFAS!F2:F6)/SUMIF(EFAS!C2:C6,"O",EFAS!D2:D6),1))</f>
         <v>—</v>
       </c>
       <c r="E18" s="268">
@@ -9726,11 +9524,10 @@
         <v>724</v>
       </c>
       <c r="C19" s="266" t="str">
-        <f>"IFAS strength rating "&amp;TEXT(SUM('IFAS '!F2:F4)/SUM('IFAS '!D2:D4),"0.0")&amp;"/5"</f>
-        <v>IFAS strength rating 4.4/5</v>
+        <f>IF(SUMIF('IFAS '!C2:C5,"S",'IFAS '!D2:D5)=0,"[NEEDS CLARIFICATION: IFAS strengths have zero total weight]","IFAS strength rating "&amp;TEXT(SUMIF('IFAS '!C2:C5,"S",'IFAS '!F2:F5)/SUMIF('IFAS '!C2:C5,"S",'IFAS '!D2:D5),"0.0")&amp;"/5")</f>
       </c>
       <c r="D19" s="267" t="str">
-        <f>IF($C$8=0,"—",ROUND(SUM('IFAS '!F2:F4)/SUM('IFAS '!D2:D4),1))</f>
+        <f>IF($C$8=0,"—",ROUND(SUMIF('IFAS '!C2:C5,"S",'IFAS '!F2:F5)/SUMIF('IFAS '!C2:C5,"S",'IFAS '!D2:D5),1))</f>
         <v>—</v>
       </c>
       <c r="E19" s="268">
@@ -9753,7 +9550,7 @@
         <v>Porter's threat 2.2/3 (inverted)</v>
       </c>
       <c r="D20" s="267" t="str">
-        <f>IF($C$8=0,"—",ROUND(6-2*'Porter''s Five Forces'!D7,1))</f>
+        <f>IF($C$8=0,"—",ROUND(7-2*'Porter''s Five Forces'!D7,1))</f>
         <v>—</v>
       </c>
       <c r="E20" s="268">
@@ -9772,8 +9569,8 @@
         <v>728</v>
       </c>
       <c r="C21" s="266" t="str">
-        <f>"EFAS "&amp;TEXT(SUM(EFAS!F2:F6),"0.0")&amp;" + IFAS "&amp;TEXT(SUM('IFAS '!F2:F5),"0.0")&amp;" blended"</f>
-        <v>EFAS 3.6 + IFAS 3.2 blended</v>
+        <f>"EFAS "&amp;TEXT(SUM(EFAS!F2:F6),"0.0")&amp;" + IFAS "&amp;TEXT(SUM('IFAS '!F2:F5),"0.0")&amp;", averaged"</f>
+        <v>EFAS 3.6 + IFAS 3.2, averaged</v>
       </c>
       <c r="D21" s="267" t="str">
         <f>IF($C$8=0,"—",ROUND((SUM(EFAS!F2:F6)+SUM('IFAS '!F2:F5))/2,1))</f>
@@ -35463,7 +35260,6 @@
     <hyperlink ref="A1" location="'PRE-BRD'!A1" display="↩ Index" xr:uid="{20FC6FF8-8B9A-4935-892A-90DA41CC8516}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <legacyDrawing r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>